<commit_message>
final update to db models for mainframes, further updates to GPU model may be necessary
</commit_message>
<xml_diff>
--- a/app/db/Kyndryl_Hardware_Data_Collection.xlsx
+++ b/app/db/Kyndryl_Hardware_Data_Collection.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="113">
   <si>
     <t>Field Name</t>
   </si>
@@ -93,6 +93,24 @@
     <t>pcf_assumptions</t>
   </si>
   <si>
+    <t>PCF Data Source</t>
+  </si>
+  <si>
+    <t>Where the PCF value was obtained (e.g., vendor report URL, internal estimate).</t>
+  </si>
+  <si>
+    <t>pcf_source</t>
+  </si>
+  <si>
+    <t>PCF Confidence Level</t>
+  </si>
+  <si>
+    <t>Data quality indicator. Valid values: 'vendor_published', 'vendor_requested', 'third_party', 'estimated', 'unavailable'.</t>
+  </si>
+  <si>
+    <t>pcf_confidence</t>
+  </si>
+  <si>
     <t>Max Power (Watts TDP)</t>
   </si>
   <si>
@@ -154,15 +172,6 @@
   </si>
   <si>
     <t>lease_term_months</t>
-  </si>
-  <si>
-    <t>Circularity Score (0-1)</t>
-  </si>
-  <si>
-    <t>Internal metric: 1.0 = Fully Recyclable/Circular.</t>
-  </si>
-  <si>
-    <t>circularity_score</t>
   </si>
   <si>
     <t>MIPS (Performance)</t>
@@ -717,7 +726,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
@@ -1068,18 +1077,18 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>1</v>
+        <v>93</v>
       </c>
       <c r="B32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>95</v>
+        <v>1</v>
       </c>
       <c r="B33" t="s">
         <v>96</v>
@@ -1101,18 +1110,18 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="B35" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C35" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>103</v>
+        <v>0</v>
       </c>
       <c r="B36" t="s">
         <v>104</v>
@@ -1130,6 +1139,17 @@
       </c>
       <c r="C37" t="s">
         <v>108</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
+        <v>109</v>
+      </c>
+      <c r="B38" t="s">
+        <v>110</v>
+      </c>
+      <c r="C38" t="s">
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -1139,24 +1159,26 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T1"/>
+  <dimension ref="A1:U1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="4" width="20.7109375" customWidth="1"/>
     <col min="5" max="5" width="31.7109375" customWidth="1"/>
     <col min="6" max="6" width="20.7109375" customWidth="1"/>
-    <col min="7" max="9" width="25.7109375" customWidth="1"/>
-    <col min="10" max="11" width="22.7109375" customWidth="1"/>
-    <col min="12" max="12" width="20.7109375" customWidth="1"/>
-    <col min="13" max="13" width="24.7109375" customWidth="1"/>
-    <col min="14" max="14" width="23.7109375" customWidth="1"/>
-    <col min="15" max="15" width="27.7109375" customWidth="1"/>
-    <col min="16" max="16" width="22.7109375" customWidth="1"/>
-    <col min="17" max="19" width="20.7109375" customWidth="1"/>
-    <col min="20" max="20" width="22.7109375" customWidth="1"/>
+    <col min="7" max="7" width="25.7109375" customWidth="1"/>
+    <col min="8" max="8" width="20.7109375" customWidth="1"/>
+    <col min="9" max="9" width="24.7109375" customWidth="1"/>
+    <col min="10" max="11" width="25.7109375" customWidth="1"/>
+    <col min="12" max="13" width="22.7109375" customWidth="1"/>
+    <col min="14" max="14" width="20.7109375" customWidth="1"/>
+    <col min="15" max="15" width="24.7109375" customWidth="1"/>
+    <col min="16" max="16" width="23.7109375" customWidth="1"/>
+    <col min="17" max="17" width="22.7109375" customWidth="1"/>
+    <col min="18" max="20" width="20.7109375" customWidth="1"/>
+    <col min="21" max="21" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20">
+    <row r="1" spans="1:21">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1216,6 +1238,9 @@
       </c>
       <c r="T1" s="1" t="s">
         <v>60</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1225,22 +1250,24 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T1"/>
+  <dimension ref="A1:U1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="4" width="20.7109375" customWidth="1"/>
     <col min="5" max="5" width="31.7109375" customWidth="1"/>
     <col min="6" max="6" width="20.7109375" customWidth="1"/>
-    <col min="7" max="9" width="25.7109375" customWidth="1"/>
-    <col min="10" max="11" width="22.7109375" customWidth="1"/>
-    <col min="12" max="12" width="20.7109375" customWidth="1"/>
-    <col min="13" max="13" width="24.7109375" customWidth="1"/>
-    <col min="14" max="14" width="23.7109375" customWidth="1"/>
-    <col min="15" max="15" width="27.7109375" customWidth="1"/>
-    <col min="16" max="20" width="20.7109375" customWidth="1"/>
+    <col min="7" max="7" width="25.7109375" customWidth="1"/>
+    <col min="8" max="8" width="20.7109375" customWidth="1"/>
+    <col min="9" max="9" width="24.7109375" customWidth="1"/>
+    <col min="10" max="11" width="25.7109375" customWidth="1"/>
+    <col min="12" max="13" width="22.7109375" customWidth="1"/>
+    <col min="14" max="14" width="20.7109375" customWidth="1"/>
+    <col min="15" max="15" width="24.7109375" customWidth="1"/>
+    <col min="16" max="16" width="23.7109375" customWidth="1"/>
+    <col min="17" max="21" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20">
+    <row r="1" spans="1:21">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1287,7 +1314,7 @@
         <v>45</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>66</v>
@@ -1300,6 +1327,9 @@
       </c>
       <c r="T1" s="1" t="s">
         <v>75</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -1309,22 +1339,24 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:T1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="4" width="20.7109375" customWidth="1"/>
     <col min="5" max="5" width="31.7109375" customWidth="1"/>
     <col min="6" max="6" width="20.7109375" customWidth="1"/>
-    <col min="7" max="9" width="25.7109375" customWidth="1"/>
-    <col min="10" max="11" width="22.7109375" customWidth="1"/>
-    <col min="12" max="12" width="20.7109375" customWidth="1"/>
-    <col min="13" max="13" width="24.7109375" customWidth="1"/>
-    <col min="14" max="14" width="23.7109375" customWidth="1"/>
-    <col min="15" max="15" width="27.7109375" customWidth="1"/>
-    <col min="16" max="19" width="20.7109375" customWidth="1"/>
+    <col min="7" max="7" width="25.7109375" customWidth="1"/>
+    <col min="8" max="8" width="20.7109375" customWidth="1"/>
+    <col min="9" max="9" width="24.7109375" customWidth="1"/>
+    <col min="10" max="11" width="25.7109375" customWidth="1"/>
+    <col min="12" max="13" width="22.7109375" customWidth="1"/>
+    <col min="14" max="14" width="20.7109375" customWidth="1"/>
+    <col min="15" max="15" width="24.7109375" customWidth="1"/>
+    <col min="16" max="16" width="23.7109375" customWidth="1"/>
+    <col min="17" max="20" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1371,7 +1403,7 @@
         <v>45</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>81</v>
@@ -1381,6 +1413,9 @@
       </c>
       <c r="S1" s="1" t="s">
         <v>87</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1403,19 +1438,19 @@
         <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1436,10 +1471,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
deleted a lot of unnecessary things
</commit_message>
<xml_diff>
--- a/app/db/Kyndryl_Hardware_Data_Collection.xlsx
+++ b/app/db/Kyndryl_Hardware_Data_Collection.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dbchristenson/Desktop/python/kyndryl-factbase/app/db/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1A7BFB3-CA0C-0049-9B2E-6A30B5D0CEC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="4440" yWindow="760" windowWidth="22580" windowHeight="17260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="READ ME - Definitions" sheetId="1" r:id="rId1"/>
@@ -14,12 +20,25 @@
     <sheet name="Vendor Programs" sheetId="5" r:id="rId5"/>
     <sheet name="Data Sources" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="116">
   <si>
     <t>Field Name</t>
   </si>
@@ -358,13 +377,22 @@
   </si>
   <si>
     <t>Program Name</t>
+  </si>
+  <si>
+    <t>IBM</t>
+  </si>
+  <si>
+    <t>z17</t>
+  </si>
+  <si>
+    <t>z-series mainframe</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -438,13 +466,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -482,7 +518,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -516,6 +552,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -550,9 +587,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -725,16 +763,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C38"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="30.7109375" customWidth="1"/>
-    <col min="2" max="2" width="65.7109375" customWidth="1"/>
-    <col min="3" max="3" width="25.7109375" customWidth="1"/>
+    <col min="1" max="1" width="30.6640625" customWidth="1"/>
+    <col min="2" max="2" width="65.6640625" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -745,7 +783,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -756,7 +794,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -767,7 +805,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -778,7 +816,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -789,7 +827,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -800,7 +838,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -811,7 +849,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -822,7 +860,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -833,7 +871,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -844,7 +882,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -855,7 +893,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>33</v>
       </c>
@@ -866,7 +904,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>36</v>
       </c>
@@ -877,7 +915,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>39</v>
       </c>
@@ -888,7 +926,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>42</v>
       </c>
@@ -899,7 +937,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>45</v>
       </c>
@@ -910,7 +948,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>48</v>
       </c>
@@ -921,7 +959,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>51</v>
       </c>
@@ -932,7 +970,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>54</v>
       </c>
@@ -943,7 +981,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>57</v>
       </c>
@@ -954,7 +992,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>60</v>
       </c>
@@ -965,7 +1003,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>63</v>
       </c>
@@ -976,7 +1014,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>66</v>
       </c>
@@ -987,7 +1025,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>69</v>
       </c>
@@ -998,7 +1036,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>72</v>
       </c>
@@ -1009,7 +1047,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>75</v>
       </c>
@@ -1020,7 +1058,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>78</v>
       </c>
@@ -1031,7 +1069,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>81</v>
       </c>
@@ -1042,7 +1080,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>84</v>
       </c>
@@ -1053,7 +1091,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="30" spans="1:3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>87</v>
       </c>
@@ -1064,7 +1102,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>90</v>
       </c>
@@ -1075,7 +1113,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>93</v>
       </c>
@@ -1086,7 +1124,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>1</v>
       </c>
@@ -1097,7 +1135,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>98</v>
       </c>
@@ -1108,7 +1146,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>101</v>
       </c>
@@ -1119,7 +1157,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>0</v>
       </c>
@@ -1130,7 +1168,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>106</v>
       </c>
@@ -1141,7 +1179,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>109</v>
       </c>
@@ -1158,27 +1196,27 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:U2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="4" width="20.7109375" customWidth="1"/>
-    <col min="5" max="5" width="31.7109375" customWidth="1"/>
-    <col min="6" max="6" width="20.7109375" customWidth="1"/>
-    <col min="7" max="7" width="25.7109375" customWidth="1"/>
-    <col min="8" max="8" width="20.7109375" customWidth="1"/>
-    <col min="9" max="9" width="24.7109375" customWidth="1"/>
-    <col min="10" max="11" width="25.7109375" customWidth="1"/>
-    <col min="12" max="13" width="22.7109375" customWidth="1"/>
-    <col min="14" max="14" width="20.7109375" customWidth="1"/>
-    <col min="15" max="15" width="24.7109375" customWidth="1"/>
-    <col min="16" max="16" width="23.7109375" customWidth="1"/>
-    <col min="17" max="17" width="22.7109375" customWidth="1"/>
-    <col min="18" max="20" width="20.7109375" customWidth="1"/>
-    <col min="21" max="21" width="22.7109375" customWidth="1"/>
+    <col min="1" max="4" width="20.6640625" customWidth="1"/>
+    <col min="5" max="5" width="31.6640625" customWidth="1"/>
+    <col min="6" max="6" width="20.6640625" customWidth="1"/>
+    <col min="7" max="7" width="25.6640625" customWidth="1"/>
+    <col min="8" max="8" width="20.6640625" customWidth="1"/>
+    <col min="9" max="9" width="24.6640625" customWidth="1"/>
+    <col min="10" max="11" width="25.6640625" customWidth="1"/>
+    <col min="12" max="13" width="22.6640625" customWidth="1"/>
+    <col min="14" max="14" width="20.6640625" customWidth="1"/>
+    <col min="15" max="15" width="24.6640625" customWidth="1"/>
+    <col min="16" max="16" width="23.6640625" customWidth="1"/>
+    <col min="17" max="17" width="22.6640625" customWidth="1"/>
+    <col min="18" max="20" width="20.6640625" customWidth="1"/>
+    <col min="21" max="21" width="22.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1241,6 +1279,20 @@
       </c>
       <c r="U1" s="1" t="s">
         <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C2">
+        <v>2024</v>
+      </c>
+      <c r="D2" t="s">
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -1249,25 +1301,25 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:U1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="4" width="20.7109375" customWidth="1"/>
-    <col min="5" max="5" width="31.7109375" customWidth="1"/>
-    <col min="6" max="6" width="20.7109375" customWidth="1"/>
-    <col min="7" max="7" width="25.7109375" customWidth="1"/>
-    <col min="8" max="8" width="20.7109375" customWidth="1"/>
-    <col min="9" max="9" width="24.7109375" customWidth="1"/>
-    <col min="10" max="11" width="25.7109375" customWidth="1"/>
-    <col min="12" max="13" width="22.7109375" customWidth="1"/>
-    <col min="14" max="14" width="20.7109375" customWidth="1"/>
-    <col min="15" max="15" width="24.7109375" customWidth="1"/>
-    <col min="16" max="16" width="23.7109375" customWidth="1"/>
-    <col min="17" max="21" width="20.7109375" customWidth="1"/>
+    <col min="1" max="4" width="20.6640625" customWidth="1"/>
+    <col min="5" max="5" width="31.6640625" customWidth="1"/>
+    <col min="6" max="6" width="20.6640625" customWidth="1"/>
+    <col min="7" max="7" width="25.6640625" customWidth="1"/>
+    <col min="8" max="8" width="20.6640625" customWidth="1"/>
+    <col min="9" max="9" width="24.6640625" customWidth="1"/>
+    <col min="10" max="11" width="25.6640625" customWidth="1"/>
+    <col min="12" max="13" width="22.6640625" customWidth="1"/>
+    <col min="14" max="14" width="20.6640625" customWidth="1"/>
+    <col min="15" max="15" width="24.6640625" customWidth="1"/>
+    <col min="16" max="16" width="23.6640625" customWidth="1"/>
+    <col min="17" max="21" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1338,25 +1390,25 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:T1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="4" width="20.7109375" customWidth="1"/>
-    <col min="5" max="5" width="31.7109375" customWidth="1"/>
-    <col min="6" max="6" width="20.7109375" customWidth="1"/>
-    <col min="7" max="7" width="25.7109375" customWidth="1"/>
-    <col min="8" max="8" width="20.7109375" customWidth="1"/>
-    <col min="9" max="9" width="24.7109375" customWidth="1"/>
-    <col min="10" max="11" width="25.7109375" customWidth="1"/>
-    <col min="12" max="13" width="22.7109375" customWidth="1"/>
-    <col min="14" max="14" width="20.7109375" customWidth="1"/>
-    <col min="15" max="15" width="24.7109375" customWidth="1"/>
-    <col min="16" max="16" width="23.7109375" customWidth="1"/>
-    <col min="17" max="20" width="20.7109375" customWidth="1"/>
+    <col min="1" max="4" width="20.6640625" customWidth="1"/>
+    <col min="5" max="5" width="31.6640625" customWidth="1"/>
+    <col min="6" max="6" width="20.6640625" customWidth="1"/>
+    <col min="7" max="7" width="25.6640625" customWidth="1"/>
+    <col min="8" max="8" width="20.6640625" customWidth="1"/>
+    <col min="9" max="9" width="24.6640625" customWidth="1"/>
+    <col min="10" max="11" width="25.6640625" customWidth="1"/>
+    <col min="12" max="13" width="22.6640625" customWidth="1"/>
+    <col min="14" max="14" width="20.6640625" customWidth="1"/>
+    <col min="15" max="15" width="24.6640625" customWidth="1"/>
+    <col min="16" max="16" width="23.6640625" customWidth="1"/>
+    <col min="17" max="20" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1424,16 +1476,16 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="4" width="20.7109375" customWidth="1"/>
-    <col min="5" max="5" width="24.7109375" customWidth="1"/>
-    <col min="6" max="6" width="26.7109375" customWidth="1"/>
+    <col min="1" max="4" width="20.6640625" customWidth="1"/>
+    <col min="5" max="5" width="24.6640625" customWidth="1"/>
+    <col min="6" max="6" width="26.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1459,14 +1511,14 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="3" width="20.7109375" customWidth="1"/>
+    <col min="1" max="3" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>

</xml_diff>